<commit_message>
Venting hole diameter and CuCrZr-IG Treatment B
</commit_message>
<xml_diff>
--- a/src/cassy/additional_data/materials/CuCrZr-IG-C.xlsx
+++ b/src/cassy/additional_data/materials/CuCrZr-IG-C.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\d.laghi\Documents\GitHub\StressAssessment\Materials\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cassy\src\cassy\additional_data\materials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8039BB2-D133-4FF2-B22B-1284E31896C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCF66749-F49E-4B14-AF08-2C2B79F07338}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="30936" windowHeight="16896" firstSheet="3" activeTab="8" xr2:uid="{FB402876-AA8B-47D7-BD9B-CC0289AC277F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="3" activeTab="6" xr2:uid="{FB402876-AA8B-47D7-BD9B-CC0289AC277F}"/>
   </bookViews>
   <sheets>
     <sheet name="Young Modulus" sheetId="2" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="24">
   <si>
     <t>T</t>
   </si>
@@ -853,7 +853,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="116">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1059,7 +1059,6 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="4" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1114,8 +1113,8 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1128,91 +1127,80 @@
     <xf numFmtId="11" fontId="7" fillId="5" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normale" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1491,14 +1479,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41A6DCC6-AA86-4E07-8334-6D45DEC2B6AE}">
   <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="6" width="8.88671875" style="2"/>
-    <col min="7" max="7" width="24.109375" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="2"/>
+    <col min="1" max="6" width="8.85546875" style="2"/>
+    <col min="7" max="7" width="24.140625" style="2" customWidth="1"/>
+    <col min="8" max="16384" width="8.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1506,7 +1494,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>-300</v>
       </c>
@@ -1514,7 +1502,7 @@
         <v>127.5</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>20</v>
       </c>
@@ -1522,7 +1510,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>100</v>
       </c>
@@ -1530,7 +1518,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>150</v>
       </c>
@@ -1544,7 +1532,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>200</v>
       </c>
@@ -1552,7 +1540,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>250</v>
       </c>
@@ -1560,7 +1548,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>300</v>
       </c>
@@ -1568,7 +1556,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>350</v>
       </c>
@@ -1576,7 +1564,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>400</v>
       </c>
@@ -1584,7 +1572,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>450</v>
       </c>
@@ -1592,7 +1580,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>500</v>
       </c>
@@ -1600,7 +1588,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>550</v>
       </c>
@@ -1608,7 +1596,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>600</v>
       </c>
@@ -1616,7 +1604,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>650</v>
       </c>
@@ -1624,7 +1612,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>700</v>
       </c>
@@ -1632,7 +1620,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
         <v>100000</v>
       </c>
@@ -1649,34 +1637,34 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E5D19D6-AC5F-4EA5-969E-16AFA5A7510C}">
   <dimension ref="A1:P5"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="8.88671875" style="2"/>
+    <col min="1" max="16384" width="8.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="36" t="s">
         <v>16</v>
       </c>
       <c r="B1" s="36"/>
-      <c r="C1" s="112" t="s">
+      <c r="C1" s="110" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="113"/>
-      <c r="E1" s="113"/>
-      <c r="F1" s="113"/>
-      <c r="G1" s="113"/>
-      <c r="H1" s="113"/>
-      <c r="I1" s="113"/>
-      <c r="J1" s="113"/>
-      <c r="K1" s="113"/>
-      <c r="L1" s="113"/>
-      <c r="M1" s="113"/>
-      <c r="N1" s="113"/>
-      <c r="O1" s="113"/>
+      <c r="D1" s="111"/>
+      <c r="E1" s="111"/>
+      <c r="F1" s="111"/>
+      <c r="G1" s="111"/>
+      <c r="H1" s="111"/>
+      <c r="I1" s="111"/>
+      <c r="J1" s="111"/>
+      <c r="K1" s="111"/>
+      <c r="L1" s="111"/>
+      <c r="M1" s="111"/>
+      <c r="N1" s="111"/>
+      <c r="O1" s="111"/>
       <c r="P1" s="37"/>
     </row>
-    <row r="2" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="38" t="s">
         <v>0</v>
       </c>
@@ -1686,7 +1674,7 @@
       <c r="C2" s="40">
         <v>100000000</v>
       </c>
-      <c r="D2" s="91">
+      <c r="D2" s="90">
         <v>150000000</v>
       </c>
       <c r="E2" s="41">
@@ -1726,153 +1714,153 @@
         <v>1000000000000</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="43">
         <v>20</v>
       </c>
       <c r="B3" s="44">
         <v>1</v>
       </c>
-      <c r="C3" s="92">
+      <c r="C3" s="91">
         <v>1</v>
       </c>
-      <c r="D3" s="93">
+      <c r="D3" s="53">
         <v>1.0009999999999999</v>
       </c>
-      <c r="E3" s="94">
+      <c r="E3" s="92">
         <v>1.0089999999999999</v>
       </c>
-      <c r="F3" s="94">
+      <c r="F3" s="92">
         <v>1.0549999999999999</v>
       </c>
-      <c r="G3" s="94">
+      <c r="G3" s="92">
         <v>1.1459999999999999</v>
       </c>
-      <c r="H3" s="94">
+      <c r="H3" s="92">
         <v>1.258</v>
       </c>
-      <c r="I3" s="94">
+      <c r="I3" s="92">
         <v>1.377</v>
       </c>
-      <c r="J3" s="94">
+      <c r="J3" s="92">
         <v>1.4990000000000001</v>
       </c>
-      <c r="K3" s="94">
+      <c r="K3" s="92">
         <v>1.6220000000000001</v>
       </c>
-      <c r="L3" s="94">
+      <c r="L3" s="92">
         <v>1.7450000000000001</v>
       </c>
-      <c r="M3" s="94">
+      <c r="M3" s="92">
         <v>1.867</v>
       </c>
-      <c r="N3" s="94">
+      <c r="N3" s="92">
         <v>1.9890000000000001</v>
       </c>
-      <c r="O3" s="94">
+      <c r="O3" s="92">
         <v>2.109</v>
       </c>
-      <c r="P3" s="95">
+      <c r="P3" s="93">
         <v>2.109</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A4" s="90">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="89">
         <v>200</v>
       </c>
       <c r="B4" s="39">
         <v>1</v>
       </c>
-      <c r="C4" s="96">
+      <c r="C4" s="94">
         <v>1</v>
       </c>
-      <c r="D4" s="97">
+      <c r="D4" s="95">
         <v>1.002</v>
       </c>
-      <c r="E4" s="98">
+      <c r="E4" s="96">
         <v>1.0269999999999999</v>
       </c>
-      <c r="F4" s="98">
+      <c r="F4" s="96">
         <v>1.111</v>
       </c>
-      <c r="G4" s="98">
+      <c r="G4" s="96">
         <v>1.2330000000000001</v>
       </c>
-      <c r="H4" s="98">
+      <c r="H4" s="96">
         <v>1.367</v>
       </c>
-      <c r="I4" s="98">
+      <c r="I4" s="96">
         <v>1.5049999999999999</v>
       </c>
-      <c r="J4" s="98">
+      <c r="J4" s="96">
         <v>1.6439999999999999</v>
       </c>
-      <c r="K4" s="98">
+      <c r="K4" s="96">
         <v>1.7829999999999999</v>
       </c>
-      <c r="L4" s="98">
+      <c r="L4" s="96">
         <v>1.921</v>
       </c>
-      <c r="M4" s="98">
+      <c r="M4" s="96">
         <v>2.0579999999999998</v>
       </c>
-      <c r="N4" s="98">
+      <c r="N4" s="96">
         <v>2.1930000000000001</v>
       </c>
-      <c r="O4" s="98">
+      <c r="O4" s="96">
         <v>2.3279999999999998</v>
       </c>
-      <c r="P4" s="95">
+      <c r="P4" s="93">
         <v>2.3279999999999998</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="45">
         <v>350</v>
       </c>
       <c r="B5" s="46">
         <v>1</v>
       </c>
-      <c r="C5" s="99">
+      <c r="C5" s="97">
         <v>1</v>
       </c>
-      <c r="D5" s="100">
+      <c r="D5" s="58">
         <v>1.008</v>
       </c>
-      <c r="E5" s="101">
+      <c r="E5" s="98">
         <v>1.0740000000000001</v>
       </c>
-      <c r="F5" s="101">
+      <c r="F5" s="98">
         <v>1.2050000000000001</v>
       </c>
-      <c r="G5" s="101">
+      <c r="G5" s="98">
         <v>1.359</v>
       </c>
-      <c r="H5" s="101">
+      <c r="H5" s="98">
         <v>1.5189999999999999</v>
       </c>
-      <c r="I5" s="101">
+      <c r="I5" s="98">
         <v>1.68</v>
       </c>
-      <c r="J5" s="101">
+      <c r="J5" s="98">
         <v>1.84</v>
       </c>
-      <c r="K5" s="101">
+      <c r="K5" s="98">
         <v>1.9990000000000001</v>
       </c>
-      <c r="L5" s="101">
+      <c r="L5" s="98">
         <v>2.1560000000000001</v>
       </c>
-      <c r="M5" s="101">
+      <c r="M5" s="98">
         <v>2.3119999999999998</v>
       </c>
-      <c r="N5" s="101">
+      <c r="N5" s="98">
         <v>2.4660000000000002</v>
       </c>
-      <c r="O5" s="101">
+      <c r="O5" s="98">
         <v>2.6190000000000002</v>
       </c>
-      <c r="P5" s="95">
+      <c r="P5" s="93">
         <v>2.6190000000000002</v>
       </c>
     </row>
@@ -1887,34 +1875,34 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05B91955-3194-42FD-9EBC-F9DC508AF353}">
   <dimension ref="A1:P5"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="8.88671875" style="2"/>
+    <col min="1" max="16384" width="8.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="36" t="s">
         <v>16</v>
       </c>
       <c r="B1" s="36"/>
-      <c r="C1" s="112" t="s">
+      <c r="C1" s="110" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="113"/>
-      <c r="E1" s="113"/>
-      <c r="F1" s="113"/>
-      <c r="G1" s="113"/>
-      <c r="H1" s="113"/>
-      <c r="I1" s="113"/>
-      <c r="J1" s="113"/>
-      <c r="K1" s="113"/>
-      <c r="L1" s="113"/>
-      <c r="M1" s="113"/>
-      <c r="N1" s="113"/>
-      <c r="O1" s="113"/>
+      <c r="D1" s="111"/>
+      <c r="E1" s="111"/>
+      <c r="F1" s="111"/>
+      <c r="G1" s="111"/>
+      <c r="H1" s="111"/>
+      <c r="I1" s="111"/>
+      <c r="J1" s="111"/>
+      <c r="K1" s="111"/>
+      <c r="L1" s="111"/>
+      <c r="M1" s="111"/>
+      <c r="N1" s="111"/>
+      <c r="O1" s="111"/>
       <c r="P1" s="37"/>
     </row>
-    <row r="2" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="38" t="s">
         <v>0</v>
       </c>
@@ -1924,7 +1912,7 @@
       <c r="C2" s="40">
         <v>100000000</v>
       </c>
-      <c r="D2" s="91">
+      <c r="D2" s="90">
         <v>150000000</v>
       </c>
       <c r="E2" s="41">
@@ -1964,153 +1952,153 @@
         <v>1000000000000</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="43">
         <v>20</v>
       </c>
       <c r="B3" s="44">
         <v>1</v>
       </c>
-      <c r="C3" s="92">
+      <c r="C3" s="91">
         <v>1</v>
       </c>
-      <c r="D3" s="93">
+      <c r="D3" s="53">
         <v>1</v>
       </c>
-      <c r="E3" s="94">
+      <c r="E3" s="92">
         <v>1.006</v>
       </c>
-      <c r="F3" s="94">
+      <c r="F3" s="92">
         <v>1.032</v>
       </c>
-      <c r="G3" s="94">
+      <c r="G3" s="92">
         <v>1.0740000000000001</v>
       </c>
-      <c r="H3" s="94">
+      <c r="H3" s="92">
         <v>1.1160000000000001</v>
       </c>
-      <c r="I3" s="94">
+      <c r="I3" s="92">
         <v>1.1519999999999999</v>
       </c>
-      <c r="J3" s="94">
+      <c r="J3" s="92">
         <v>1.1830000000000001</v>
       </c>
-      <c r="K3" s="94">
+      <c r="K3" s="92">
         <v>1.21</v>
       </c>
-      <c r="L3" s="94">
+      <c r="L3" s="92">
         <v>1.232</v>
       </c>
-      <c r="M3" s="94">
+      <c r="M3" s="92">
         <v>1.2509999999999999</v>
       </c>
-      <c r="N3" s="94">
+      <c r="N3" s="92">
         <v>1.268</v>
       </c>
-      <c r="O3" s="94">
+      <c r="O3" s="92">
         <v>1.2829999999999999</v>
       </c>
-      <c r="P3" s="95">
+      <c r="P3" s="93">
         <v>1.2829999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A4" s="90">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="89">
         <v>200</v>
       </c>
       <c r="B4" s="39">
         <v>1</v>
       </c>
-      <c r="C4" s="96">
+      <c r="C4" s="94">
         <v>1</v>
       </c>
-      <c r="D4" s="97">
+      <c r="D4" s="95">
         <v>1.0009999999999999</v>
       </c>
-      <c r="E4" s="98">
+      <c r="E4" s="96">
         <v>1.0169999999999999</v>
       </c>
-      <c r="F4" s="98">
+      <c r="F4" s="96">
         <v>1.0589999999999999</v>
       </c>
-      <c r="G4" s="98">
+      <c r="G4" s="96">
         <v>1.107</v>
       </c>
-      <c r="H4" s="98">
+      <c r="H4" s="96">
         <v>1.149</v>
       </c>
-      <c r="I4" s="98">
+      <c r="I4" s="96">
         <v>1.1850000000000001</v>
       </c>
-      <c r="J4" s="98">
+      <c r="J4" s="96">
         <v>1.214</v>
       </c>
-      <c r="K4" s="98">
+      <c r="K4" s="96">
         <v>1.238</v>
       </c>
-      <c r="L4" s="98">
+      <c r="L4" s="96">
         <v>1.2589999999999999</v>
       </c>
-      <c r="M4" s="98">
+      <c r="M4" s="96">
         <v>1.2769999999999999</v>
       </c>
-      <c r="N4" s="98">
+      <c r="N4" s="96">
         <v>1.292</v>
       </c>
-      <c r="O4" s="98">
+      <c r="O4" s="96">
         <v>1.306</v>
       </c>
-      <c r="P4" s="95">
+      <c r="P4" s="93">
         <v>1.306</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="45">
         <v>350</v>
       </c>
       <c r="B5" s="46">
         <v>1</v>
       </c>
-      <c r="C5" s="99">
+      <c r="C5" s="97">
         <v>1</v>
       </c>
-      <c r="D5" s="100">
+      <c r="D5" s="58">
         <v>1.0049999999999999</v>
       </c>
-      <c r="E5" s="101">
+      <c r="E5" s="98">
         <v>1.0409999999999999</v>
       </c>
-      <c r="F5" s="101">
+      <c r="F5" s="98">
         <v>1.097</v>
       </c>
-      <c r="G5" s="101">
+      <c r="G5" s="98">
         <v>1.147</v>
       </c>
-      <c r="H5" s="101">
+      <c r="H5" s="98">
         <v>1.1879999999999999</v>
       </c>
-      <c r="I5" s="101">
+      <c r="I5" s="98">
         <v>1.2210000000000001</v>
       </c>
-      <c r="J5" s="101">
+      <c r="J5" s="98">
         <v>1.2470000000000001</v>
       </c>
-      <c r="K5" s="101">
+      <c r="K5" s="98">
         <v>1.27</v>
       </c>
-      <c r="L5" s="101">
+      <c r="L5" s="98">
         <v>1.288</v>
       </c>
-      <c r="M5" s="101">
+      <c r="M5" s="98">
         <v>1.304</v>
       </c>
-      <c r="N5" s="101">
+      <c r="N5" s="98">
         <v>1.3180000000000001</v>
       </c>
-      <c r="O5" s="101">
+      <c r="O5" s="98">
         <v>1.33</v>
       </c>
-      <c r="P5" s="95">
+      <c r="P5" s="93">
         <v>1.33</v>
       </c>
     </row>
@@ -2125,13 +2113,13 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{174D964C-7EB0-4B95-AE83-97098D6EB823}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="12.33203125" style="2" customWidth="1"/>
-    <col min="3" max="16384" width="8.88671875" style="2"/>
+    <col min="1" max="2" width="12.28515625" style="2" customWidth="1"/>
+    <col min="3" max="16384" width="8.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="47" t="s">
         <v>0</v>
       </c>
@@ -2142,7 +2130,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="49">
         <v>-300</v>
       </c>
@@ -2153,7 +2141,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="52">
         <v>20</v>
       </c>
@@ -2164,7 +2152,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="55">
         <v>200</v>
       </c>
@@ -2175,7 +2163,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="56">
         <v>350</v>
       </c>
@@ -2186,7 +2174,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="57">
         <v>500</v>
       </c>
@@ -2197,7 +2185,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="60">
         <v>100000</v>
       </c>
@@ -2216,17 +2204,17 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5CA0493-D284-4DEE-B058-7FF56E305F20}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0.3</v>
       </c>
@@ -2239,50 +2227,50 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48DAB5F6-9D7E-4BA9-ADCC-0FE2BE75E93E}">
   <dimension ref="A1:H15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="8.88671875" style="5"/>
+    <col min="1" max="16384" width="8.85546875" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="114" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="109" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="114"/>
-      <c r="C1" s="114"/>
-      <c r="D1" s="114"/>
-      <c r="E1" s="114"/>
-      <c r="F1" s="114"/>
-      <c r="G1" s="114"/>
-      <c r="H1" s="114"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="B3" s="111" t="s">
+      <c r="B1" s="109"/>
+      <c r="C1" s="109"/>
+      <c r="D1" s="109"/>
+      <c r="E1" s="109"/>
+      <c r="F1" s="109"/>
+      <c r="G1" s="109"/>
+      <c r="H1" s="109"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B3" s="108" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="111"/>
-      <c r="D3" s="111"/>
-      <c r="E3" s="111"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="102" t="s">
+      <c r="C3" s="108"/>
+      <c r="D3" s="108"/>
+      <c r="E3" s="108"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="102">
+      <c r="B4" s="32">
         <v>0</v>
       </c>
-      <c r="C4" s="102">
+      <c r="C4" s="32">
         <v>0.29999900000000002</v>
       </c>
-      <c r="D4" s="102">
+      <c r="D4" s="32">
         <v>0.3</v>
       </c>
-      <c r="E4" s="102">
+      <c r="E4" s="32">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="102">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="32">
         <v>20</v>
       </c>
       <c r="B5" s="5">
@@ -2292,8 +2280,8 @@
         <v>10.9</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="102">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="32">
         <v>50</v>
       </c>
       <c r="B6" s="5">
@@ -2303,8 +2291,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="102">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="32">
         <v>100</v>
       </c>
       <c r="B7" s="5">
@@ -2320,8 +2308,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="102">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="32">
         <v>150</v>
       </c>
       <c r="B8" s="5">
@@ -2337,8 +2325,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="102">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="32">
         <v>200</v>
       </c>
       <c r="B9" s="5">
@@ -2354,8 +2342,8 @@
         <v>0.17</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="102">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="32">
         <v>250</v>
       </c>
       <c r="B10" s="5">
@@ -2371,8 +2359,8 @@
         <v>3.16</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="102">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="32">
         <v>300</v>
       </c>
       <c r="B11" s="5">
@@ -2388,8 +2376,8 @@
         <v>7.35</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="102">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="32">
         <v>350</v>
       </c>
       <c r="B12" s="5">
@@ -2405,8 +2393,8 @@
         <v>11.28</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" s="102">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="32">
         <v>400</v>
       </c>
       <c r="B13" s="5">
@@ -2416,8 +2404,8 @@
         <v>5.8</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A14" s="102">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="32">
         <v>450</v>
       </c>
       <c r="B14" s="5">
@@ -2427,8 +2415,8 @@
         <v>6.2</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" s="102">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="32">
         <v>500</v>
       </c>
       <c r="B15" s="5">
@@ -2451,12 +2439,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69A4A868-0133-454B-AECC-B1A432929753}">
   <dimension ref="A1:C19"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="8.88671875" style="5"/>
+    <col min="1" max="16384" width="8.85546875" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>2</v>
       </c>
@@ -2464,23 +2452,23 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="43.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="103" t="s">
+    <row r="2" spans="1:3" ht="43.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="100" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="103"/>
-      <c r="C2" s="103"/>
-    </row>
-    <row r="3" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="100"/>
+      <c r="C2" s="100"/>
+    </row>
+    <row r="3" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="104" t="s">
+      <c r="B3" s="101" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="105"/>
-    </row>
-    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C3" s="102"/>
+    </row>
+    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>6</v>
       </c>
@@ -2491,7 +2479,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="10">
         <v>10</v>
       </c>
@@ -2502,7 +2490,7 @@
         <v>2.5529999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="13">
         <v>20</v>
       </c>
@@ -2513,7 +2501,7 @@
         <v>2.552</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="13">
         <v>40</v>
       </c>
@@ -2524,7 +2512,7 @@
         <v>1.931</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="63">
         <v>100</v>
       </c>
@@ -2535,7 +2523,7 @@
         <v>1.4850000000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="63">
         <v>200</v>
       </c>
@@ -2546,7 +2534,7 @@
         <v>1.08</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="63">
         <v>400</v>
       </c>
@@ -2557,7 +2545,7 @@
         <v>0.86899999999999999</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="63">
         <v>1000</v>
       </c>
@@ -2568,7 +2556,7 @@
         <v>0.71499999999999997</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="63">
         <v>2000</v>
       </c>
@@ -2579,7 +2567,7 @@
         <v>0.57799999999999996</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="63">
         <v>4000</v>
       </c>
@@ -2590,7 +2578,7 @@
         <v>0.48799999999999999</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="63">
         <v>10000</v>
       </c>
@@ -2601,7 +2589,7 @@
         <v>0.41199999999999998</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="63">
         <v>100000</v>
       </c>
@@ -2612,7 +2600,7 @@
         <v>0.33</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="63">
         <v>200000</v>
       </c>
@@ -2623,7 +2611,7 @@
         <v>0.28199999999999997</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="63">
         <v>400000</v>
       </c>
@@ -2634,7 +2622,7 @@
         <v>0.249</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="63">
         <v>1000000</v>
       </c>
@@ -2645,7 +2633,7 @@
         <v>0.221</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="15">
         <v>100000000</v>
       </c>
@@ -2669,26 +2657,26 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACC1B8EB-9779-49C3-9702-6E2647BB475F}">
   <dimension ref="A1:H14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="10.88671875" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="106" t="s">
+    <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="103" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="107"/>
-      <c r="C1" s="108"/>
-    </row>
-    <row r="2" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B1" s="104"/>
+      <c r="C1" s="105"/>
+    </row>
+    <row r="2" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="16"/>
-      <c r="B2" s="109" t="s">
+      <c r="B2" s="106" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="110"/>
-    </row>
-    <row r="3" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C2" s="107"/>
+    </row>
+    <row r="3" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="17" t="s">
         <v>9</v>
       </c>
@@ -2699,7 +2687,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="20">
         <v>20</v>
       </c>
@@ -2710,7 +2698,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="23">
         <v>50</v>
       </c>
@@ -2721,7 +2709,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="26">
         <v>100</v>
       </c>
@@ -2732,7 +2720,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="26">
         <v>150</v>
       </c>
@@ -2743,7 +2731,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="26">
         <v>200</v>
       </c>
@@ -2755,7 +2743,7 @@
       </c>
       <c r="H8" s="29"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="26">
         <v>250</v>
       </c>
@@ -2766,7 +2754,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="26">
         <v>300</v>
       </c>
@@ -2777,7 +2765,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="26">
         <v>350</v>
       </c>
@@ -2788,7 +2776,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="26">
         <v>400</v>
       </c>
@@ -2799,7 +2787,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="26">
         <v>450</v>
       </c>
@@ -2810,7 +2798,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="65">
         <v>500</v>
       </c>
@@ -2834,34 +2822,34 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{597EBE28-BB6B-4425-B68F-E12DBD3E3E4F}">
   <dimension ref="A1:L14"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="5"/>
+    <col min="1" max="1" width="8.85546875" style="5"/>
     <col min="2" max="2" width="9" style="5" customWidth="1"/>
-    <col min="3" max="16384" width="8.88671875" style="5"/>
+    <col min="3" max="16384" width="8.85546875" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="32" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B2" s="111" t="s">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B2" s="108" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="111"/>
-      <c r="D2" s="111"/>
-      <c r="E2" s="111"/>
-      <c r="F2" s="111"/>
-      <c r="G2" s="111"/>
-      <c r="H2" s="111"/>
-      <c r="I2" s="111"/>
-      <c r="J2" s="111"/>
-      <c r="K2" s="111"/>
-      <c r="L2" s="111"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C2" s="108"/>
+      <c r="D2" s="108"/>
+      <c r="E2" s="108"/>
+      <c r="F2" s="108"/>
+      <c r="G2" s="108"/>
+      <c r="H2" s="108"/>
+      <c r="I2" s="108"/>
+      <c r="J2" s="108"/>
+      <c r="K2" s="108"/>
+      <c r="L2" s="108"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="32" t="s">
         <v>9</v>
       </c>
@@ -2881,7 +2869,7 @@
       <c r="K3" s="32"/>
       <c r="L3" s="32"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="33">
         <v>20</v>
       </c>
@@ -2892,7 +2880,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="32">
         <v>50</v>
       </c>
@@ -2903,7 +2891,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="32">
         <v>100</v>
       </c>
@@ -2914,7 +2902,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="32">
         <v>150</v>
       </c>
@@ -2925,7 +2913,7 @@
         <v>1.46</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="32">
         <v>200</v>
       </c>
@@ -2936,7 +2924,7 @@
         <v>1.49</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="32">
         <v>250</v>
       </c>
@@ -2947,7 +2935,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="32">
         <v>300</v>
       </c>
@@ -2958,7 +2946,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="32">
         <v>350</v>
       </c>
@@ -2969,7 +2957,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
         <v>400</v>
       </c>
@@ -2980,7 +2968,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
         <v>450</v>
       </c>
@@ -2991,7 +2979,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
         <v>500</v>
       </c>
@@ -3014,24 +3002,24 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24335452-4334-459A-9143-079A47F85124}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="13.33203125" style="5" customWidth="1"/>
-    <col min="3" max="16384" width="8.88671875" style="5"/>
+    <col min="1" max="2" width="13.28515625" style="5" customWidth="1"/>
+    <col min="3" max="16384" width="8.85546875" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B2" s="111" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B2" s="108" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="111"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C2" s="108"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="32" t="s">
         <v>9</v>
       </c>
@@ -3042,7 +3030,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
         <v>20</v>
       </c>
@@ -3053,7 +3041,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
         <v>50</v>
       </c>
@@ -3064,7 +3052,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>100</v>
       </c>
@@ -3075,7 +3063,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>150</v>
       </c>
@@ -3086,7 +3074,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
         <v>200</v>
       </c>
@@ -3097,7 +3085,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
         <v>250</v>
       </c>
@@ -3108,7 +3096,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
         <v>300</v>
       </c>
@@ -3119,7 +3107,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
         <v>350</v>
       </c>
@@ -3130,7 +3118,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
         <v>400</v>
       </c>
@@ -3141,7 +3129,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
         <v>450</v>
       </c>
@@ -3152,7 +3140,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
         <v>500</v>
       </c>
@@ -3175,152 +3163,152 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{708A983D-881C-4742-B17E-B3A9A7EA90E7}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.5546875" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="34"/>
-      <c r="B2" s="111" t="s">
+      <c r="B2" s="108" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="111"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="70" t="s">
+      <c r="C2" s="108"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="69" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="81">
+      <c r="B3" s="80">
         <v>0</v>
       </c>
-      <c r="C3" s="82">
+      <c r="C3" s="81">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="78">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="77">
         <v>20</v>
       </c>
-      <c r="B4" s="83">
+      <c r="B4" s="82">
         <v>296</v>
       </c>
-      <c r="C4" s="84">
+      <c r="C4" s="83">
         <v>296</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="78">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="77">
         <v>50</v>
       </c>
-      <c r="B5" s="83">
+      <c r="B5" s="82">
         <v>296</v>
       </c>
-      <c r="C5" s="84">
+      <c r="C5" s="83">
         <v>296</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="78">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="77">
         <v>100</v>
       </c>
-      <c r="B6" s="83">
+      <c r="B6" s="82">
         <v>394</v>
       </c>
-      <c r="C6" s="84">
+      <c r="C6" s="83">
         <v>394</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="78">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="77">
         <v>150</v>
       </c>
-      <c r="B7" s="83">
+      <c r="B7" s="82">
         <v>492</v>
       </c>
-      <c r="C7" s="84">
+      <c r="C7" s="83">
         <v>492</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="78">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="77">
         <v>200</v>
       </c>
-      <c r="B8" s="68" t="s">
+      <c r="B8" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="74" t="s">
+      <c r="C8" s="73" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="78">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="77">
         <v>250</v>
       </c>
-      <c r="B9" s="68" t="s">
+      <c r="B9" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="74" t="s">
+      <c r="C9" s="73" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="78">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="77">
         <v>300</v>
       </c>
-      <c r="B10" s="68" t="s">
+      <c r="B10" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="74" t="s">
+      <c r="C10" s="73" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="78">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="77">
         <v>350</v>
       </c>
-      <c r="B11" s="68" t="s">
+      <c r="B11" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="74" t="s">
+      <c r="C11" s="73" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="79">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="78">
         <v>400</v>
       </c>
-      <c r="B12" s="69" t="s">
+      <c r="B12" s="68" t="s">
         <v>15</v>
       </c>
-      <c r="C12" s="75" t="s">
+      <c r="C12" s="74" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="79">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="78">
         <v>450</v>
       </c>
-      <c r="B13" s="69" t="s">
+      <c r="B13" s="68" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="75" t="s">
+      <c r="C13" s="74" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="80">
+    <row r="14" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="79">
         <v>500</v>
       </c>
-      <c r="B14" s="76" t="s">
+      <c r="B14" s="75" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="77" t="s">
+      <c r="C14" s="76" t="s">
         <v>15</v>
       </c>
     </row>
@@ -3335,149 +3323,149 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{934453F1-6A59-45D3-8BB5-EACDE123E36C}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="34"/>
-      <c r="B2" s="111" t="s">
+      <c r="B2" s="108" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="111"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="70" t="s">
+      <c r="C2" s="108"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="69" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="81">
+      <c r="B3" s="80">
         <v>0</v>
       </c>
-      <c r="C3" s="82">
+      <c r="C3" s="81">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="78">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="77">
         <v>20</v>
       </c>
-      <c r="B4" s="83">
+      <c r="B4" s="82">
         <v>241</v>
       </c>
-      <c r="C4" s="84">
+      <c r="C4" s="83">
         <v>241</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="78">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="77">
         <v>50</v>
       </c>
-      <c r="B5" s="83">
+      <c r="B5" s="82">
+        <v>241</v>
+      </c>
+      <c r="C5" s="83">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="77">
+        <v>100</v>
+      </c>
+      <c r="B6" s="82">
         <v>237</v>
       </c>
-      <c r="C5" s="84">
+      <c r="C6" s="83">
         <v>237</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="78">
-        <v>100</v>
-      </c>
-      <c r="B6" s="83">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="77">
+        <v>150</v>
+      </c>
+      <c r="B7" s="82">
         <v>235</v>
       </c>
-      <c r="C6" s="84">
+      <c r="C7" s="83">
         <v>235</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="78">
-        <v>150</v>
-      </c>
-      <c r="B7" s="83">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="77">
+        <v>200</v>
+      </c>
+      <c r="B8" s="82">
         <v>223</v>
       </c>
-      <c r="C7" s="84">
+      <c r="C8" s="83">
         <v>223</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="78">
-        <v>200</v>
-      </c>
-      <c r="B8" s="83">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="77">
+        <v>250</v>
+      </c>
+      <c r="B9" s="82">
         <v>421</v>
       </c>
-      <c r="C8" s="84">
+      <c r="C9" s="83">
         <v>421</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="78">
-        <v>250</v>
-      </c>
-      <c r="B9" s="83">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="77">
+        <v>300</v>
+      </c>
+      <c r="B10" s="82">
         <v>727</v>
       </c>
-      <c r="C9" s="84">
+      <c r="C10" s="83">
         <v>727</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="78">
-        <v>300</v>
-      </c>
-      <c r="B10" s="68" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="77">
+        <v>350</v>
+      </c>
+      <c r="B11" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="74" t="s">
+      <c r="C11" s="73" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="78">
-        <v>350</v>
-      </c>
-      <c r="B11" s="68" t="s">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="78">
+        <v>400</v>
+      </c>
+      <c r="B12" s="68" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="74" t="s">
+      <c r="C12" s="74" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="79">
-        <v>400</v>
-      </c>
-      <c r="B12" s="69" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="78">
+        <v>450</v>
+      </c>
+      <c r="B13" s="68" t="s">
         <v>15</v>
       </c>
-      <c r="C12" s="75" t="s">
+      <c r="C13" s="74" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="79">
-        <v>450</v>
-      </c>
-      <c r="B13" s="69" t="s">
+    <row r="14" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="79">
+        <v>500</v>
+      </c>
+      <c r="B14" s="75" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="75" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="80">
-        <v>500</v>
-      </c>
-      <c r="B14" s="76" t="s">
-        <v>15</v>
-      </c>
-      <c r="C14" s="77" t="s">
+      <c r="C14" s="76" t="s">
         <v>15</v>
       </c>
     </row>
@@ -3492,98 +3480,98 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74160366-A75D-4B56-8711-C6A1795D1C47}">
   <dimension ref="A1:AW14"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="8.88671875" style="5"/>
+    <col min="1" max="16384" width="8.85546875" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="A1" s="111" t="s">
+    <row r="1" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A1" s="108" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="111"/>
-      <c r="C1" s="111"/>
-      <c r="D1" s="111"/>
-      <c r="E1" s="111"/>
-      <c r="F1" s="111"/>
-      <c r="G1" s="111"/>
-      <c r="H1" s="111"/>
-      <c r="I1" s="111"/>
-      <c r="J1" s="111"/>
-      <c r="K1" s="111"/>
-      <c r="L1" s="111"/>
-      <c r="M1" s="111"/>
-      <c r="N1" s="111"/>
-      <c r="O1" s="111"/>
-    </row>
-    <row r="2" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="B2" s="111" t="s">
+      <c r="B1" s="108"/>
+      <c r="C1" s="108"/>
+      <c r="D1" s="108"/>
+      <c r="E1" s="108"/>
+      <c r="F1" s="108"/>
+      <c r="G1" s="108"/>
+      <c r="H1" s="108"/>
+      <c r="I1" s="108"/>
+      <c r="J1" s="108"/>
+      <c r="K1" s="108"/>
+      <c r="L1" s="108"/>
+      <c r="M1" s="108"/>
+      <c r="N1" s="108"/>
+      <c r="O1" s="108"/>
+    </row>
+    <row r="2" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="B2" s="108" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="111"/>
-      <c r="D2" s="111"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="67"/>
-      <c r="L2" s="67"/>
-      <c r="M2" s="67"/>
-      <c r="N2" s="67"/>
-      <c r="O2" s="67"/>
-      <c r="P2" s="67"/>
-      <c r="Q2" s="67"/>
-      <c r="R2" s="67"/>
-      <c r="S2" s="67"/>
-      <c r="T2" s="67"/>
-      <c r="U2" s="67"/>
-      <c r="V2" s="67"/>
-      <c r="W2" s="67"/>
-      <c r="X2" s="67"/>
-      <c r="Y2" s="67"/>
-      <c r="Z2" s="67"/>
-      <c r="AA2" s="67"/>
-      <c r="AB2" s="67"/>
-      <c r="AC2" s="67"/>
-      <c r="AD2" s="67"/>
-      <c r="AE2" s="67"/>
-      <c r="AF2" s="67"/>
-      <c r="AG2" s="67"/>
-      <c r="AH2" s="67"/>
-      <c r="AI2" s="67"/>
-      <c r="AJ2" s="67"/>
-      <c r="AK2" s="67"/>
-      <c r="AL2" s="67"/>
-      <c r="AM2" s="67"/>
-      <c r="AN2" s="67"/>
-      <c r="AO2" s="67"/>
-      <c r="AP2" s="67"/>
-      <c r="AQ2" s="67"/>
-      <c r="AR2" s="67"/>
-      <c r="AS2" s="67"/>
-      <c r="AT2" s="67"/>
-      <c r="AU2" s="67"/>
-      <c r="AV2" s="67"/>
-      <c r="AW2" s="67"/>
-    </row>
-    <row r="3" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="A3" s="102" t="s">
+      <c r="C2" s="108"/>
+      <c r="D2" s="108"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
+      <c r="J2" s="34"/>
+      <c r="K2" s="34"/>
+      <c r="L2" s="34"/>
+      <c r="M2" s="34"/>
+      <c r="N2" s="34"/>
+      <c r="O2" s="34"/>
+      <c r="P2" s="34"/>
+      <c r="Q2" s="34"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
+      <c r="T2" s="34"/>
+      <c r="U2" s="34"/>
+      <c r="V2" s="34"/>
+      <c r="W2" s="34"/>
+      <c r="X2" s="34"/>
+      <c r="Y2" s="34"/>
+      <c r="Z2" s="34"/>
+      <c r="AA2" s="34"/>
+      <c r="AB2" s="34"/>
+      <c r="AC2" s="34"/>
+      <c r="AD2" s="34"/>
+      <c r="AE2" s="34"/>
+      <c r="AF2" s="34"/>
+      <c r="AG2" s="34"/>
+      <c r="AH2" s="34"/>
+      <c r="AI2" s="34"/>
+      <c r="AJ2" s="34"/>
+      <c r="AK2" s="34"/>
+      <c r="AL2" s="34"/>
+      <c r="AM2" s="34"/>
+      <c r="AN2" s="34"/>
+      <c r="AO2" s="34"/>
+      <c r="AP2" s="34"/>
+      <c r="AQ2" s="34"/>
+      <c r="AR2" s="34"/>
+      <c r="AS2" s="34"/>
+      <c r="AT2" s="34"/>
+      <c r="AU2" s="34"/>
+      <c r="AV2" s="34"/>
+      <c r="AW2" s="34"/>
+    </row>
+    <row r="3" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A3" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="102">
+      <c r="B3" s="32">
         <v>0</v>
       </c>
-      <c r="C3" s="102">
+      <c r="C3" s="32">
         <v>1E-3</v>
       </c>
-      <c r="D3" s="102">
+      <c r="D3" s="32">
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="A4" s="102">
+    <row r="4" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A4" s="32">
         <v>20</v>
       </c>
       <c r="B4" s="5">
@@ -3596,8 +3584,8 @@
         <v>319</v>
       </c>
     </row>
-    <row r="5" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="A5" s="102">
+    <row r="5" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A5" s="32">
         <v>50</v>
       </c>
       <c r="B5" s="5">
@@ -3610,8 +3598,8 @@
         <v>319</v>
       </c>
     </row>
-    <row r="6" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="A6" s="102">
+    <row r="6" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A6" s="32">
         <v>100</v>
       </c>
       <c r="B6" s="5">
@@ -3624,8 +3612,8 @@
         <v>319</v>
       </c>
     </row>
-    <row r="7" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="A7" s="102">
+    <row r="7" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A7" s="32">
         <v>150</v>
       </c>
       <c r="B7" s="5">
@@ -3638,8 +3626,8 @@
         <v>300</v>
       </c>
     </row>
-    <row r="8" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="A8" s="102">
+    <row r="8" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A8" s="32">
         <v>200</v>
       </c>
       <c r="B8" s="5">
@@ -3652,8 +3640,8 @@
         <v>292</v>
       </c>
     </row>
-    <row r="9" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="A9" s="102">
+    <row r="9" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A9" s="32">
         <v>250</v>
       </c>
       <c r="B9" s="5">
@@ -3666,8 +3654,8 @@
         <v>255</v>
       </c>
     </row>
-    <row r="10" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="A10" s="102">
+    <row r="10" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A10" s="32">
         <v>300</v>
       </c>
       <c r="B10" s="5">
@@ -3680,8 +3668,8 @@
         <v>218</v>
       </c>
     </row>
-    <row r="11" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="A11" s="102">
+    <row r="11" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A11" s="32">
         <v>350</v>
       </c>
       <c r="B11" s="5">
@@ -3694,8 +3682,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="A12" s="102">
+    <row r="12" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A12" s="32">
         <v>400</v>
       </c>
       <c r="B12" s="5">
@@ -3708,8 +3696,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="A13" s="102">
+    <row r="13" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A13" s="32">
         <v>450</v>
       </c>
       <c r="B13" s="5">
@@ -3722,8 +3710,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:49" x14ac:dyDescent="0.3">
-      <c r="A14" s="102">
+    <row r="14" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A14" s="32">
         <v>500</v>
       </c>
       <c r="B14" s="5">
@@ -3749,48 +3737,48 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BBB63CF-CFA2-4F00-8D7F-2DA9D07B46E3}">
   <dimension ref="A1:I14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="13.77734375" customWidth="1"/>
+    <col min="3" max="3" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="114" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="109" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="114"/>
-      <c r="C1" s="114"/>
-      <c r="D1" s="114"/>
-      <c r="E1" s="114"/>
-      <c r="F1" s="114"/>
-      <c r="G1" s="114"/>
-      <c r="H1" s="114"/>
-      <c r="I1" s="114"/>
-    </row>
-    <row r="2" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B1" s="109"/>
+      <c r="C1" s="109"/>
+      <c r="D1" s="109"/>
+      <c r="E1" s="109"/>
+      <c r="F1" s="109"/>
+      <c r="G1" s="109"/>
+      <c r="H1" s="109"/>
+      <c r="I1" s="109"/>
+    </row>
+    <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="34"/>
-      <c r="B2" s="111" t="s">
+      <c r="B2" s="108" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="111"/>
-      <c r="D2" s="111"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="70" t="s">
+      <c r="C2" s="108"/>
+      <c r="D2" s="108"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="69" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="71">
+      <c r="B3" s="70">
         <v>0</v>
       </c>
-      <c r="C3" s="89">
+      <c r="C3" s="88">
         <v>1E-3</v>
       </c>
-      <c r="D3" s="72">
+      <c r="D3" s="71">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="85">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="84">
         <v>20</v>
       </c>
       <c r="B4" s="64" t="s">
@@ -3799,12 +3787,12 @@
       <c r="C4" s="64">
         <v>106.33333333333333</v>
       </c>
-      <c r="D4" s="73">
+      <c r="D4" s="72">
         <v>106.33333333333333</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="85">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="84">
         <v>50</v>
       </c>
       <c r="B5" s="64" t="s">
@@ -3813,12 +3801,12 @@
       <c r="C5" s="64">
         <v>106.33333333333333</v>
       </c>
-      <c r="D5" s="73">
+      <c r="D5" s="72">
         <v>106.33333333333333</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="85">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="84">
         <v>100</v>
       </c>
       <c r="B6" s="64" t="s">
@@ -3827,12 +3815,12 @@
       <c r="C6" s="64">
         <v>106.33333333333333</v>
       </c>
-      <c r="D6" s="73">
+      <c r="D6" s="72">
         <v>106.33333333333333</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="85">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="84">
         <v>150</v>
       </c>
       <c r="B7" s="64" t="s">
@@ -3841,12 +3829,12 @@
       <c r="C7" s="64">
         <v>100</v>
       </c>
-      <c r="D7" s="73">
+      <c r="D7" s="72">
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" s="85">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="84">
         <v>200</v>
       </c>
       <c r="B8" s="64" t="s">
@@ -3855,12 +3843,12 @@
       <c r="C8" s="64">
         <v>98.180333333333323</v>
       </c>
-      <c r="D8" s="73">
+      <c r="D8" s="72">
         <v>98.180333333333323</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="85">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="84">
         <v>250</v>
       </c>
       <c r="B9" s="64" t="s">
@@ -3869,12 +3857,12 @@
       <c r="C9" s="64">
         <v>100.52683333333334</v>
       </c>
-      <c r="D9" s="73">
+      <c r="D9" s="72">
         <v>100.52683333333334</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="85">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="84">
         <v>300</v>
       </c>
       <c r="B10" s="64" t="s">
@@ -3883,12 +3871,12 @@
       <c r="C10" s="64">
         <v>108.18199999999999</v>
       </c>
-      <c r="D10" s="73">
+      <c r="D10" s="72">
         <v>108.18199999999999</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="85">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="84">
         <v>350</v>
       </c>
       <c r="B11" s="64" t="s">
@@ -3897,12 +3885,12 @@
       <c r="C11" s="64" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="73" t="s">
+      <c r="D11" s="72" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="86">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="85">
         <v>400</v>
       </c>
       <c r="B12" s="64" t="s">
@@ -3911,12 +3899,12 @@
       <c r="C12" s="64" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="73" t="s">
+      <c r="D12" s="72" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="86">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="85">
         <v>450</v>
       </c>
       <c r="B13" s="64" t="s">
@@ -3925,21 +3913,21 @@
       <c r="C13" s="64" t="s">
         <v>15</v>
       </c>
-      <c r="D13" s="73" t="s">
+      <c r="D13" s="72" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="87">
+    <row r="14" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="86">
         <v>500</v>
       </c>
-      <c r="B14" s="88" t="s">
+      <c r="B14" s="87" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="88" t="s">
+      <c r="C14" s="87" t="s">
         <v>15</v>
       </c>
-      <c r="D14" s="115" t="s">
+      <c r="D14" s="99" t="s">
         <v>15</v>
       </c>
     </row>
@@ -3954,6 +3942,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100EFE0C39B20CFE747B2EDBEF1A424A9C1" ma:contentTypeVersion="14" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="fc5d43efe255f0326fdf88779d9e8cc0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="71e126cb-1963-4e7b-b13a-15d2f64f78e9" xmlns:ns3="f41f4605-e15c-4135-bd96-d3970596b173" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c67b044c92a952204dd5da40bf3ff3c1" ns2:_="" ns3:_="">
     <xsd:import namespace="71e126cb-1963-4e7b-b13a-15d2f64f78e9"/>
@@ -4182,15 +4179,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -4203,13 +4191,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D596418F-2539-4C91-ADDD-9ACDDCB72504}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8943BE27-877E-487E-BD20-6C08F78D6224}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8943BE27-877E-487E-BD20-6C08F78D6224}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D596418F-2539-4C91-ADDD-9ACDDCB72504}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="71e126cb-1963-4e7b-b13a-15d2f64f78e9"/>
+    <ds:schemaRef ds:uri="f41f4605-e15c-4135-bd96-d3970596b173"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E565C311-B736-4044-9BB9-4FAF6430CAF6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E565C311-B736-4044-9BB9-4FAF6430CAF6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="f41f4605-e15c-4135-bd96-d3970596b173"/>
+    <ds:schemaRef ds:uri="71e126cb-1963-4e7b-b13a-15d2f64f78e9"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>